<commit_message>
Started polishing the plots. Multistability in 2D tested successfully. Frequency oscillators tested but remain to be seen if they were successfull.
</commit_message>
<xml_diff>
--- a/apps_results_MAK_REINFORCE/RPA_3species_5rxns/RPA_3species_5rxns_MAK_REINFORCE.xlsx
+++ b/apps_results_MAK_REINFORCE/RPA_3species_5rxns/RPA_3species_5rxns_MAK_REINFORCE.xlsx
@@ -10,14 +10,14 @@
     <sheet r:id="rId1" sheetId="1" name="Data"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Data'!$A$1:$W$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">=Data!$A$1:$W$4</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="40">
   <si>
     <t>Timestamp</t>
   </si>
@@ -88,10 +88,10 @@
     <t>Structure Head Temperature</t>
   </si>
   <si>
-    <t>2025-11-23 08:20:45</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/5fcb25657f444095bdac6517214d322b</t>
+    <t>2025-11-23 12:31:07</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/db72f20d328e4db08c9e633179816629</t>
   </si>
   <si>
     <t>Yes*</t>
@@ -100,10 +100,10 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>Fixed bug: weighing the topk vs remaining entropies. Convergence was very fast, and topological diversity was high.</t>
-  </si>
-  <si>
-    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 2.0, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+    <t xml:space="preserve">Increased the entropy weight of the structure head from 2 to 2.5. Good run similar to the good one before. </t>
+  </si>
+  <si>
+    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 2.5, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
   </si>
   <si>
     <t>0.0001</t>
@@ -119,48 +119,6 @@
   </si>
   <si>
     <t>{'target_entropy_ratio_to_max': np.float64(0.35679185088982296), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
-  </si>
-  <si>
-    <t>2025-11-23 10:20:28</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/6e9dbdc7f666497d89225f2c2b861ffa</t>
-  </si>
-  <si>
-    <t>Yes/No</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conditions are the same as the previous run. Fast convergence (not as fast as before), but topological diversity is low. Entropy of the batch deviated from the entropy of the topk at the end which means that diversifying started happening without getting good topologies. </t>
-  </si>
-  <si>
-    <t>2025-11-23 10:51:52</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/eb0ad05d9cd146ee983662d71d0e5f89</t>
-  </si>
-  <si>
-    <t>Conditions are the same as the previous run. Good convergence speed (a little slower than before), and topological diversity is high.</t>
-  </si>
-  <si>
-    <t>2025-11-23 11:28:45</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/b217d90512dd438d8a5a4adc434dac6f</t>
-  </si>
-  <si>
-    <t>Conditions are the same as the previous run. Good convergence speed. Modest diversity in topologies.</t>
-  </si>
-  <si>
-    <t>2025-11-23 12:31:07</t>
-  </si>
-  <si>
-    <t>https://www.comet.com/maurice-filo/rpa-3species-5rxns-mak-reinforce/db72f20d328e4db08c9e633179816629</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Increased the entropy weight of the structure head from 2 to 2.5. Good run similar to the good one before. </t>
-  </si>
-  <si>
-    <t>{'entropy_weight': 0.001, 'entropy_weight_structure_head': 2.5, 'entropy_weight_continuous_head': 1.0, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
   </si>
   <si>
     <t>2025-11-23 13:06:31</t>
@@ -186,7 +144,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -197,12 +155,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -234,15 +186,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -553,35 +502,35 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:W8"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="4" width="20.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="11.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="4" width="6.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="4" width="273.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="4" width="254.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="4" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="5" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="4" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="5" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="5" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="5" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="5" width="7.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="4" width="74.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="5" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="5" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="5" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="5" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="5" width="21.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="5" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="4" width="25.005" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="4" width="134.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="3" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="3" width="49.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="3" width="11.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="3" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="3" width="6.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="3" width="273.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="3" width="254.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="3" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="4" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="3" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="4" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="4" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="4" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="4" width="7.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="3" width="74.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="4" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="4" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="4" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="4" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="4" width="21.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="4" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="3" width="25.005" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="3" width="134.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -652,7 +601,7 @@
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1" t="s">
         <v>23</v>
       </c>
@@ -723,7 +672,7 @@
         <v>33</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
@@ -731,7 +680,7 @@
         <v>35</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>26</v>
@@ -740,7 +689,7 @@
         <v>26</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>28</v>
@@ -794,12 +743,12 @@
         <v>33</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>25</v>
@@ -811,7 +760,7 @@
         <v>26</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>28</v>
@@ -862,284 +811,6 @@
         <v>32</v>
       </c>
       <c r="W4" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I5" s="2">
-        <v>300</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K5" s="2">
-        <v>5</v>
-      </c>
-      <c r="L5" s="2">
-        <v>1024</v>
-      </c>
-      <c r="M5" s="2">
-        <v>10240</v>
-      </c>
-      <c r="N5" s="2">
-        <v>128</v>
-      </c>
-      <c r="O5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P5" s="2">
-        <v>10</v>
-      </c>
-      <c r="Q5" s="2">
-        <v>30</v>
-      </c>
-      <c r="R5" s="2">
-        <v>100</v>
-      </c>
-      <c r="S5" s="2">
-        <v>1000</v>
-      </c>
-      <c r="T5" s="2">
-        <v>1</v>
-      </c>
-      <c r="U5" s="2">
-        <v>9</v>
-      </c>
-      <c r="V5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W5" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I6" s="2">
-        <v>300</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K6" s="2">
-        <v>5</v>
-      </c>
-      <c r="L6" s="2">
-        <v>1024</v>
-      </c>
-      <c r="M6" s="2">
-        <v>10240</v>
-      </c>
-      <c r="N6" s="2">
-        <v>128</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P6" s="2">
-        <v>10</v>
-      </c>
-      <c r="Q6" s="2">
-        <v>30</v>
-      </c>
-      <c r="R6" s="2">
-        <v>100</v>
-      </c>
-      <c r="S6" s="2">
-        <v>1000</v>
-      </c>
-      <c r="T6" s="2">
-        <v>1</v>
-      </c>
-      <c r="U6" s="2">
-        <v>9</v>
-      </c>
-      <c r="V6" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W6" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I7" s="2">
-        <v>300</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K7" s="2">
-        <v>5</v>
-      </c>
-      <c r="L7" s="2">
-        <v>1024</v>
-      </c>
-      <c r="M7" s="2">
-        <v>10240</v>
-      </c>
-      <c r="N7" s="2">
-        <v>128</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P7" s="2">
-        <v>10</v>
-      </c>
-      <c r="Q7" s="2">
-        <v>30</v>
-      </c>
-      <c r="R7" s="2">
-        <v>100</v>
-      </c>
-      <c r="S7" s="2">
-        <v>1000</v>
-      </c>
-      <c r="T7" s="2">
-        <v>1</v>
-      </c>
-      <c r="U7" s="2">
-        <v>9</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W7" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
-      <c r="A8" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I8" s="3">
-        <v>300</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K8" s="3">
-        <v>5</v>
-      </c>
-      <c r="L8" s="3">
-        <v>1024</v>
-      </c>
-      <c r="M8" s="3">
-        <v>10240</v>
-      </c>
-      <c r="N8" s="3">
-        <v>128</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P8" s="3">
-        <v>10</v>
-      </c>
-      <c r="Q8" s="3">
-        <v>30</v>
-      </c>
-      <c r="R8" s="3">
-        <v>100</v>
-      </c>
-      <c r="S8" s="3">
-        <v>1000</v>
-      </c>
-      <c r="T8" s="3">
-        <v>1</v>
-      </c>
-      <c r="U8" s="3">
-        <v>9</v>
-      </c>
-      <c r="V8" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W8" s="1" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>